<commit_message>
updated excell sheet with both amazon and flipkart datasets analysis
</commit_message>
<xml_diff>
--- a/docs/dataset_audit.xlsx
+++ b/docs/dataset_audit.xlsx
@@ -8,12 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Vivek\Documents\projectda\CartIQQ\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A6E6ADD5-D96D-4AB6-A976-B02EB1ACBE61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5034880A-501A-4086-B23D-D0432FEBDBC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{4EEF50C5-A59C-4A80-B14A-EEF719768441}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Dataset Summary" sheetId="1" r:id="rId1"/>
+    <sheet name="Column comparison" sheetId="2" r:id="rId2"/>
+    <sheet name="Missing Values" sheetId="4" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -34,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="35">
   <si>
     <t>Feature</t>
   </si>
@@ -45,16 +47,10 @@
     <t>Flipkart</t>
   </si>
   <si>
-    <t>Rows</t>
-  </si>
-  <si>
-    <t>Columns</t>
-  </si>
-  <si>
     <t>Product Name column</t>
   </si>
   <si>
-    <t>Brand column</t>
+    <t>Category column</t>
   </si>
   <si>
     <t>Price column</t>
@@ -70,19 +66,112 @@
   </si>
   <si>
     <t>Data types</t>
+  </si>
+  <si>
+    <t>product_name</t>
+  </si>
+  <si>
+    <t>actual_price</t>
+  </si>
+  <si>
+    <t>rating</t>
+  </si>
+  <si>
+    <t>str</t>
+  </si>
+  <si>
+    <t>np.int64(0)</t>
+  </si>
+  <si>
+    <t>rating_count 2</t>
+  </si>
+  <si>
+    <t>Number of Rows</t>
+  </si>
+  <si>
+    <t>Number of Columns</t>
+  </si>
+  <si>
+    <t>Review count column</t>
+  </si>
+  <si>
+    <t>category</t>
+  </si>
+  <si>
+    <t>price</t>
+  </si>
+  <si>
+    <t>rating_count</t>
+  </si>
+  <si>
+    <t>StandardName</t>
+  </si>
+  <si>
+    <t>Column</t>
+  </si>
+  <si>
+    <t>Rating</t>
+  </si>
+  <si>
+    <t>Discount</t>
+  </si>
+  <si>
+    <t>retail_price</t>
+  </si>
+  <si>
+    <t>product_rating</t>
+  </si>
+  <si>
+    <t>retail_price 78
+discounted_price 78
+image 3
+description 2
+brand 5864
+product_specifications 14</t>
+  </si>
+  <si>
+    <t>str,float64,bool</t>
+  </si>
+  <si>
+    <t>overall_rating</t>
+  </si>
+  <si>
+    <t>overall_count</t>
+  </si>
+  <si>
+    <t>product_category_tree</t>
+  </si>
+  <si>
+    <t>review_count</t>
+  </si>
+  <si>
+    <t>Brand</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <color theme="1"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="8"/>
+      <color theme="1"/>
+      <name val="Consolas"/>
+      <family val="3"/>
     </font>
   </fonts>
   <fills count="2">
@@ -105,8 +194,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -421,10 +519,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5E34CF27-177D-4D57-B91E-DD5BA2B2122A}">
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="35.77734375" customWidth="1"/>
+    <col min="2" max="2" width="17.6640625" customWidth="1"/>
+    <col min="3" max="3" width="22" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
@@ -440,53 +540,236 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>3</v>
+        <v>16</v>
       </c>
       <c r="B2">
         <v>1465</v>
       </c>
+      <c r="C2">
+        <v>20000</v>
+      </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="B3">
         <v>16</v>
       </c>
+      <c r="C3">
+        <v>15</v>
+      </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>5</v>
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>6</v>
+        <v>5</v>
+      </c>
+      <c r="B5" t="s">
+        <v>11</v>
+      </c>
+      <c r="C5" t="s">
+        <v>26</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C6" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" ht="100.8" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>8</v>
+      <c r="B7" t="s">
+        <v>15</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>28</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>9</v>
+        <v>8</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C8" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>10</v>
+        <v>9</v>
+      </c>
+      <c r="B9" t="s">
+        <v>13</v>
+      </c>
+      <c r="C9" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
+        <v>4</v>
+      </c>
+      <c r="B10" t="s">
+        <v>19</v>
+      </c>
+      <c r="C10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>18</v>
+      </c>
+      <c r="B11" t="s">
+        <v>21</v>
+      </c>
+      <c r="C11" t="s">
+        <v>30</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B6A1B1A1-C106-4693-99AE-8CC6078564CB}">
+  <dimension ref="A1:C5"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="24.44140625" customWidth="1"/>
+    <col min="2" max="2" width="23.5546875" customWidth="1"/>
+    <col min="3" max="3" width="22.6640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
         <v>11</v>
+      </c>
+      <c r="B3" t="s">
+        <v>26</v>
+      </c>
+      <c r="C3" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B4" t="s">
+        <v>31</v>
+      </c>
+      <c r="C4" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>19</v>
+      </c>
+      <c r="B5" t="s">
+        <v>32</v>
+      </c>
+      <c r="C5" t="s">
+        <v>19</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3C7B460D-855B-4941-850F-EE9254C6A14F}">
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B2">
+        <v>0</v>
+      </c>
+      <c r="C2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B3">
+        <v>0</v>
+      </c>
+      <c r="C3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>34</v>
+      </c>
+      <c r="B4">
+        <v>0</v>
+      </c>
+      <c r="C4">
+        <v>5864</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
finally excell sheet with coloured headers
</commit_message>
<xml_diff>
--- a/docs/dataset_audit.xlsx
+++ b/docs/dataset_audit.xlsx
@@ -345,12 +345,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="33">
+  <fills count="34">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -669,7 +675,7 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -693,16 +699,16 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
@@ -711,91 +717,91 @@
     <xf numFmtId="0" fontId="18" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
   <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -886,7 +892,7 @@
         <a:srgbClr val="E7E6E6"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4472C4"/>
+        <a:srgbClr val="5B9BD5"/>
       </a:accent1>
       <a:accent2>
         <a:srgbClr val="ED7D31"/>
@@ -898,7 +904,7 @@
         <a:srgbClr val="FFC000"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="5B9BD5"/>
+        <a:srgbClr val="4472C4"/>
       </a:accent5>
       <a:accent6>
         <a:srgbClr val="70AD47"/>

</xml_diff>